<commit_message>
Removed campground from dropdown list
</commit_message>
<xml_diff>
--- a/Commercial_Assessment_MC_2.0.xlsx
+++ b/Commercial_Assessment_MC_2.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\model\project_level_analysis\PIA_Tool_Test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amcclary\Documents\GitHub\PIA_Web_Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED4E92A1-2C30-4147-9254-6BF8D56DF7A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D45813C-75AE-4778-986A-12185F19F619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{5C0E9020-961F-4B95-A886-A07748039AB8}"/>
+    <workbookView xWindow="28680" yWindow="525" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{5C0E9020-961F-4B95-A886-A07748039AB8}"/>
   </bookViews>
   <sheets>
     <sheet name="LA" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">LA!$A$1:$K$111</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -426,7 +426,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1898" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1894" uniqueCount="378">
   <si>
     <t>LA Types</t>
   </si>
@@ -1653,7 +1653,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -1667,7 +1667,6 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1707,9 +1706,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1747,7 +1746,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1853,7 +1852,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1995,7 +1994,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2144,15 +2143,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{172908BE-441B-425E-A4F7-108BAC91D0DC}">
   <dimension ref="A1:J111"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="38.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="42.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="42.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>157</v>
       </c>
@@ -2181,7 +2180,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>159</v>
       </c>
@@ -2210,7 +2209,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>160</v>
       </c>
@@ -2239,7 +2238,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>161</v>
       </c>
@@ -2268,7 +2267,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>162</v>
       </c>
@@ -2297,7 +2296,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>163</v>
       </c>
@@ -2326,7 +2325,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>164</v>
       </c>
@@ -2355,7 +2354,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>165</v>
       </c>
@@ -2384,7 +2383,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>166</v>
       </c>
@@ -2413,7 +2412,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>167</v>
       </c>
@@ -2442,7 +2441,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>168</v>
       </c>
@@ -2468,7 +2467,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>169</v>
       </c>
@@ -2497,7 +2496,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>170</v>
       </c>
@@ -2526,7 +2525,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>171</v>
       </c>
@@ -2555,7 +2554,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>172</v>
       </c>
@@ -2584,7 +2583,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>173</v>
       </c>
@@ -2613,7 +2612,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>174</v>
       </c>
@@ -2642,7 +2641,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>175</v>
       </c>
@@ -2671,7 +2670,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>176</v>
       </c>
@@ -2700,7 +2699,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>177</v>
       </c>
@@ -2729,7 +2728,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>178</v>
       </c>
@@ -2758,7 +2757,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>179</v>
       </c>
@@ -2787,7 +2786,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>180</v>
       </c>
@@ -2816,7 +2815,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>181</v>
       </c>
@@ -2845,7 +2844,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>182</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>183</v>
       </c>
@@ -2900,7 +2899,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>184</v>
       </c>
@@ -2929,7 +2928,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>185</v>
       </c>
@@ -2958,7 +2957,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>186</v>
       </c>
@@ -2987,7 +2986,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>187</v>
       </c>
@@ -3016,7 +3015,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>188</v>
       </c>
@@ -3045,7 +3044,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -3074,7 +3073,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>190</v>
       </c>
@@ -3103,7 +3102,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>191</v>
       </c>
@@ -3129,7 +3128,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E35" t="s">
         <v>225</v>
       </c>
@@ -3146,7 +3145,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E36" t="s">
         <v>226</v>
       </c>
@@ -3163,7 +3162,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E37" t="s">
         <v>227</v>
       </c>
@@ -3180,7 +3179,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E38" t="s">
         <v>228</v>
       </c>
@@ -3197,7 +3196,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E39" t="s">
         <v>229</v>
       </c>
@@ -3214,7 +3213,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E40" t="s">
         <v>230</v>
       </c>
@@ -3228,7 +3227,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E41" t="s">
         <v>231</v>
       </c>
@@ -3245,7 +3244,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>232</v>
       </c>
@@ -3262,7 +3261,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>233</v>
       </c>
@@ -3279,7 +3278,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>234</v>
       </c>
@@ -3296,7 +3295,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E45" t="s">
         <v>235</v>
       </c>
@@ -3313,7 +3312,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
         <v>236</v>
       </c>
@@ -3330,7 +3329,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E47" t="s">
         <v>237</v>
       </c>
@@ -3347,7 +3346,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
         <v>238</v>
       </c>
@@ -3364,7 +3363,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="49" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>239</v>
       </c>
@@ -3381,7 +3380,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="50" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E50" t="s">
         <v>240</v>
       </c>
@@ -3398,7 +3397,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="51" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E51" t="s">
         <v>241</v>
       </c>
@@ -3415,7 +3414,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="52" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>242</v>
       </c>
@@ -3432,7 +3431,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="53" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E53" t="s">
         <v>243</v>
       </c>
@@ -3449,7 +3448,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="54" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>244</v>
       </c>
@@ -3466,7 +3465,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>245</v>
       </c>
@@ -3483,7 +3482,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="56" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>246</v>
       </c>
@@ -3500,7 +3499,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="57" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>247</v>
       </c>
@@ -3517,7 +3516,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>248</v>
       </c>
@@ -3534,7 +3533,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="59" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E59" t="s">
         <v>249</v>
       </c>
@@ -3551,7 +3550,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="60" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E60" t="s">
         <v>250</v>
       </c>
@@ -3568,7 +3567,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="62" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E62" t="s">
         <v>252</v>
       </c>
@@ -3585,7 +3584,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="63" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E63" t="s">
         <v>253</v>
       </c>
@@ -3602,7 +3601,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="64" spans="5:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="5:9" x14ac:dyDescent="0.25">
       <c r="E64" t="s">
         <v>254</v>
       </c>
@@ -3619,7 +3618,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="65" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
         <v>255</v>
       </c>
@@ -3636,7 +3635,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="66" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
         <v>256</v>
       </c>
@@ -3653,7 +3652,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="67" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
         <v>257</v>
       </c>
@@ -3670,7 +3669,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="68" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
         <v>258</v>
       </c>
@@ -3687,7 +3686,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="69" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E69" t="s">
         <v>259</v>
       </c>
@@ -3704,7 +3703,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="70" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E70" t="s">
         <v>260</v>
       </c>
@@ -3721,7 +3720,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="71" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E71" t="s">
         <v>261</v>
       </c>
@@ -3738,7 +3737,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="72" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E72" t="s">
         <v>262</v>
       </c>
@@ -3755,7 +3754,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="73" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
         <v>263</v>
       </c>
@@ -3772,7 +3771,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="74" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
         <v>264</v>
       </c>
@@ -3789,7 +3788,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="75" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="75" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E75" t="s">
         <v>265</v>
       </c>
@@ -3806,7 +3805,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="76" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="76" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E76" t="s">
         <v>266</v>
       </c>
@@ -3820,7 +3819,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="77" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="77" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E77" t="s">
         <v>267</v>
       </c>
@@ -3837,7 +3836,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="78" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
         <v>268</v>
       </c>
@@ -3857,7 +3856,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="79" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E79" t="s">
         <v>269</v>
       </c>
@@ -3877,7 +3876,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="80" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E80" t="s">
         <v>270</v>
       </c>
@@ -3897,7 +3896,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="81" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E81" t="s">
         <v>271</v>
       </c>
@@ -3917,7 +3916,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="82" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E82" t="s">
         <v>272</v>
       </c>
@@ -3937,7 +3936,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="83" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E83" t="s">
         <v>273</v>
       </c>
@@ -3957,7 +3956,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="84" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E84" t="s">
         <v>274</v>
       </c>
@@ -3977,7 +3976,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="85" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E85" t="s">
         <v>275</v>
       </c>
@@ -3997,7 +3996,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="86" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E86" t="s">
         <v>276</v>
       </c>
@@ -4014,7 +4013,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="87" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E87" t="s">
         <v>277</v>
       </c>
@@ -4034,7 +4033,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="88" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E88" t="s">
         <v>278</v>
       </c>
@@ -4054,7 +4053,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="89" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E89" t="s">
         <v>279</v>
       </c>
@@ -4074,7 +4073,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="90" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E90" t="s">
         <v>280</v>
       </c>
@@ -4094,7 +4093,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="91" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E91" t="s">
         <v>281</v>
       </c>
@@ -4114,7 +4113,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="92" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E92" t="s">
         <v>282</v>
       </c>
@@ -4134,7 +4133,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="93" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="93" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E93" t="s">
         <v>283</v>
       </c>
@@ -4154,7 +4153,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="94" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="94" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E94" t="s">
         <v>284</v>
       </c>
@@ -4174,7 +4173,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="95" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="95" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E95" t="s">
         <v>285</v>
       </c>
@@ -4194,7 +4193,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="96" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="96" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E96" t="s">
         <v>286</v>
       </c>
@@ -4214,7 +4213,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="97" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="97" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E97" t="s">
         <v>287</v>
       </c>
@@ -4234,7 +4233,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="98" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="98" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E98" t="s">
         <v>288</v>
       </c>
@@ -4254,7 +4253,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="99" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="99" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E99" t="s">
         <v>289</v>
       </c>
@@ -4271,7 +4270,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="100" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="100" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E100" t="s">
         <v>290</v>
       </c>
@@ -4291,7 +4290,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="101" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="101" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E101" t="s">
         <v>291</v>
       </c>
@@ -4308,7 +4307,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="102" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="102" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E102" t="s">
         <v>292</v>
       </c>
@@ -4325,7 +4324,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="103" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="103" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E103" t="s">
         <v>293</v>
       </c>
@@ -4345,7 +4344,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="104" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="104" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E104" t="s">
         <v>294</v>
       </c>
@@ -4365,7 +4364,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="105" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="105" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E105" t="s">
         <v>295</v>
       </c>
@@ -4385,7 +4384,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="106" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="106" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E106" t="s">
         <v>296</v>
       </c>
@@ -4405,7 +4404,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="107" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="107" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E107" t="s">
         <v>297</v>
       </c>
@@ -4425,7 +4424,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="108" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="108" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
         <v>298</v>
       </c>
@@ -4445,7 +4444,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="109" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="109" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E109" t="s">
         <v>299</v>
       </c>
@@ -4465,7 +4464,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="110" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="110" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E110" t="s">
         <v>300</v>
       </c>
@@ -4485,7 +4484,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="111" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="111" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
         <v>301</v>
       </c>
@@ -4501,29 +4500,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{428D2166-0D63-423B-8897-ACFF6CB5B597}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -4536,21 +4535,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16B8F70-9C0E-430C-AC9A-2F92A013F2C8}">
   <dimension ref="A1:J117"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.88671875" customWidth="1"/>
-    <col min="2" max="2" width="23.33203125" customWidth="1"/>
-    <col min="3" max="3" width="6.6640625" customWidth="1"/>
+    <col min="1" max="1" width="6.85546875" customWidth="1"/>
+    <col min="2" max="2" width="23.28515625" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="8" max="8" width="11.109375" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:10" s="3" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>159</v>
       </c>
@@ -4577,7 +4576,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E3" t="s">
         <v>207</v>
       </c>
@@ -4597,7 +4596,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>161</v>
       </c>
@@ -4629,7 +4628,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>160</v>
       </c>
@@ -4658,7 +4657,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>203</v>
       </c>
@@ -4678,7 +4677,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E7" t="s">
         <v>204</v>
       </c>
@@ -4698,7 +4697,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>162</v>
       </c>
@@ -4718,7 +4717,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>163</v>
       </c>
@@ -4738,7 +4737,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>164</v>
       </c>
@@ -4767,7 +4766,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>165</v>
       </c>
@@ -4787,7 +4786,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>166</v>
       </c>
@@ -4816,7 +4815,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E13" t="s">
         <v>251</v>
       </c>
@@ -4836,12 +4835,12 @@
         <v>209</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="5" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="16" spans="1:10" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A16" s="4" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>167</v>
       </c>
@@ -4870,7 +4869,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
         <v>212</v>
       </c>
@@ -4890,7 +4889,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E19" t="s">
         <v>213</v>
       </c>
@@ -4910,7 +4909,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E20" t="s">
         <v>215</v>
       </c>
@@ -4930,7 +4929,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>168</v>
       </c>
@@ -4959,7 +4958,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
         <v>205</v>
       </c>
@@ -4979,7 +4978,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
         <v>210</v>
       </c>
@@ -4999,12 +4998,12 @@
         <v>211</v>
       </c>
     </row>
-    <row r="26" spans="1:10" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="26" spans="1:10" s="9" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A26" s="8" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>169</v>
       </c>
@@ -5021,7 +5020,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E28" t="s">
         <v>271</v>
       </c>
@@ -5041,7 +5040,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E29" t="s">
         <v>272</v>
       </c>
@@ -5061,7 +5060,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E30" t="s">
         <v>273</v>
       </c>
@@ -5081,7 +5080,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E31" t="s">
         <v>275</v>
       </c>
@@ -5101,7 +5100,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E32" t="s">
         <v>276</v>
       </c>
@@ -5121,7 +5120,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E33" t="s">
         <v>289</v>
       </c>
@@ -5141,7 +5140,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E34" t="s">
         <v>285</v>
       </c>
@@ -5161,7 +5160,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>170</v>
       </c>
@@ -5190,7 +5189,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>171</v>
       </c>
@@ -5219,7 +5218,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -5248,7 +5247,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E38" t="s">
         <v>284</v>
       </c>
@@ -5268,7 +5267,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>173</v>
       </c>
@@ -5297,7 +5296,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>175</v>
       </c>
@@ -5326,7 +5325,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>176</v>
       </c>
@@ -5355,7 +5354,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E42" t="s">
         <v>296</v>
       </c>
@@ -5375,7 +5374,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E43" t="s">
         <v>300</v>
       </c>
@@ -5395,7 +5394,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E44" t="s">
         <v>295</v>
       </c>
@@ -5415,7 +5414,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>177</v>
       </c>
@@ -5444,7 +5443,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E46" t="s">
         <v>294</v>
       </c>
@@ -5461,7 +5460,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>178</v>
       </c>
@@ -5490,7 +5489,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E48" t="s">
         <v>281</v>
       </c>
@@ -5510,7 +5509,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E49" t="s">
         <v>282</v>
       </c>
@@ -5530,7 +5529,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>179</v>
       </c>
@@ -5559,7 +5558,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>180</v>
       </c>
@@ -5591,7 +5590,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E52" t="s">
         <v>270</v>
       </c>
@@ -5608,7 +5607,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>182</v>
       </c>
@@ -5637,7 +5636,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E54" t="s">
         <v>255</v>
       </c>
@@ -5657,7 +5656,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E55" t="s">
         <v>256</v>
       </c>
@@ -5677,7 +5676,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E56" t="s">
         <v>257</v>
       </c>
@@ -5697,7 +5696,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E57" t="s">
         <v>263</v>
       </c>
@@ -5717,7 +5716,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E58" t="s">
         <v>264</v>
       </c>
@@ -5737,14 +5736,14 @@
         <v>254</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>183</v>
       </c>
       <c r="B59" t="s">
         <v>25</v>
       </c>
-      <c r="C59" s="11">
+      <c r="C59">
         <v>720</v>
       </c>
       <c r="D59" t="s">
@@ -5766,7 +5765,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E60" t="s">
         <v>252</v>
       </c>
@@ -5786,7 +5785,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E61" t="s">
         <v>253</v>
       </c>
@@ -5806,7 +5805,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>184</v>
       </c>
@@ -5823,7 +5822,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>185</v>
       </c>
@@ -5843,7 +5842,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>186</v>
       </c>
@@ -5860,7 +5859,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
         <v>265</v>
       </c>
@@ -5880,7 +5879,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E66" t="s">
         <v>266</v>
       </c>
@@ -5894,7 +5893,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E67" t="s">
         <v>267</v>
       </c>
@@ -5908,7 +5907,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E68" t="s">
         <v>277</v>
       </c>
@@ -5925,7 +5924,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E69" t="s">
         <v>278</v>
       </c>
@@ -5945,7 +5944,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E70" t="s">
         <v>279</v>
       </c>
@@ -5965,7 +5964,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E71" t="s">
         <v>286</v>
       </c>
@@ -5985,7 +5984,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E72" t="s">
         <v>287</v>
       </c>
@@ -6005,7 +6004,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E73" t="s">
         <v>288</v>
       </c>
@@ -6025,7 +6024,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E74" t="s">
         <v>291</v>
       </c>
@@ -6045,12 +6044,12 @@
         <v>320</v>
       </c>
     </row>
-    <row r="77" spans="1:10" s="7" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="77" spans="1:10" s="7" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A77" s="6" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E78" t="s">
         <v>216</v>
       </c>
@@ -6064,7 +6063,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E79" t="s">
         <v>217</v>
       </c>
@@ -6084,7 +6083,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E80" t="s">
         <v>218</v>
       </c>
@@ -6104,7 +6103,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E81" t="s">
         <v>219</v>
       </c>
@@ -6124,7 +6123,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E82" t="s">
         <v>220</v>
       </c>
@@ -6144,7 +6143,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E83" t="s">
         <v>221</v>
       </c>
@@ -6161,7 +6160,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E84" t="s">
         <v>222</v>
       </c>
@@ -6178,7 +6177,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E85" t="s">
         <v>223</v>
       </c>
@@ -6195,7 +6194,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E86" t="s">
         <v>224</v>
       </c>
@@ -6209,7 +6208,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E87" t="s">
         <v>225</v>
       </c>
@@ -6226,7 +6225,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E88" t="s">
         <v>226</v>
       </c>
@@ -6243,7 +6242,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>181</v>
       </c>
@@ -6272,7 +6271,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E90" t="s">
         <v>228</v>
       </c>
@@ -6292,7 +6291,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E91" t="s">
         <v>229</v>
       </c>
@@ -6312,7 +6311,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E92" t="s">
         <v>230</v>
       </c>
@@ -6329,7 +6328,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E93" t="s">
         <v>231</v>
       </c>
@@ -6349,7 +6348,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>174</v>
       </c>
@@ -6378,7 +6377,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E95" t="s">
         <v>233</v>
       </c>
@@ -6398,7 +6397,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E96" t="s">
         <v>234</v>
       </c>
@@ -6415,12 +6414,12 @@
         <v>317</v>
       </c>
     </row>
-    <row r="97" spans="1:10" s="16" customFormat="1" ht="28.8" x14ac:dyDescent="0.55000000000000004">
-      <c r="A97" s="17" t="s">
+    <row r="97" spans="1:10" s="15" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A97" s="16" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>187</v>
       </c>
@@ -6449,7 +6448,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>188</v>
       </c>
@@ -6478,7 +6477,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>189</v>
       </c>
@@ -6507,7 +6506,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>190</v>
       </c>
@@ -6536,7 +6535,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E102" t="s">
         <v>240</v>
       </c>
@@ -6556,7 +6555,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E103" t="s">
         <v>238</v>
       </c>
@@ -6576,7 +6575,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>191</v>
       </c>
@@ -6605,7 +6604,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E105" t="s">
         <v>241</v>
       </c>
@@ -6625,7 +6624,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E106" t="s">
         <v>242</v>
       </c>
@@ -6645,7 +6644,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E107" t="s">
         <v>244</v>
       </c>
@@ -6662,7 +6661,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E108" t="s">
         <v>245</v>
       </c>
@@ -6682,7 +6681,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E109" t="s">
         <v>246</v>
       </c>
@@ -6702,7 +6701,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E110" t="s">
         <v>247</v>
       </c>
@@ -6719,7 +6718,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E111" t="s">
         <v>248</v>
       </c>
@@ -6736,7 +6735,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="E112" t="s">
         <v>249</v>
       </c>
@@ -6753,7 +6752,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="113" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="113" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E113" t="s">
         <v>250</v>
       </c>
@@ -6770,7 +6769,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="114" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="114" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E114" t="s">
         <v>259</v>
       </c>
@@ -6790,7 +6789,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="115" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="115" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E115" t="s">
         <v>260</v>
       </c>
@@ -6810,7 +6809,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="116" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="116" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E116" t="s">
         <v>261</v>
       </c>
@@ -6830,7 +6829,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="117" spans="5:10" x14ac:dyDescent="0.3">
+    <row r="117" spans="5:10" x14ac:dyDescent="0.25">
       <c r="E117" t="s">
         <v>262</v>
       </c>
@@ -6860,16 +6859,16 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E71DCBC4-1FA2-4664-BF09-FAF9F3DA6B88}">
   <dimension ref="A1:H52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.109375" customWidth="1"/>
-    <col min="3" max="3" width="38.44140625" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.88671875" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>350</v>
       </c>
@@ -6889,8 +6888,8 @@
         <v>347</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+    <row r="2" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B2" s="17" t="s">
         <v>331</v>
       </c>
       <c r="C2" s="3"/>
@@ -6900,7 +6899,7 @@
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -6910,7 +6909,7 @@
       <c r="C3" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3">
         <v>210</v>
       </c>
       <c r="E3">
@@ -6920,7 +6919,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -6930,7 +6929,7 @@
       <c r="C4" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="11">
+      <c r="D4">
         <v>220</v>
       </c>
       <c r="E4">
@@ -6940,7 +6939,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -6950,7 +6949,7 @@
       <c r="C5" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="11">
+      <c r="D5">
         <v>252</v>
       </c>
       <c r="E5">
@@ -6960,7 +6959,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -6970,7 +6969,7 @@
       <c r="C6" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="11">
+      <c r="D6">
         <v>253</v>
       </c>
       <c r="E6">
@@ -6980,8 +6979,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B7" s="12" t="s">
+    <row r="7" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B7" s="11" t="s">
         <v>327</v>
       </c>
       <c r="C7" s="5"/>
@@ -6991,7 +6990,7 @@
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -7011,7 +7010,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -7031,7 +7030,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>7</v>
       </c>
@@ -7051,8 +7050,8 @@
         <v>344</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B11" s="13" t="s">
+    <row r="11" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B11" s="12" t="s">
         <v>328</v>
       </c>
       <c r="C11" s="9"/>
@@ -7062,7 +7061,7 @@
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -7072,7 +7071,7 @@
       <c r="C12" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="11">
+      <c r="D12">
         <v>820</v>
       </c>
       <c r="E12">
@@ -7085,7 +7084,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -7095,7 +7094,7 @@
       <c r="C13" t="s">
         <v>148</v>
       </c>
-      <c r="D13" s="11">
+      <c r="D13">
         <v>890</v>
       </c>
       <c r="E13">
@@ -7105,7 +7104,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -7115,7 +7114,7 @@
       <c r="C14" t="s">
         <v>146</v>
       </c>
-      <c r="D14" s="11">
+      <c r="D14">
         <v>880</v>
       </c>
       <c r="E14">
@@ -7125,7 +7124,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -7135,7 +7134,7 @@
       <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="11">
+      <c r="D15">
         <v>850</v>
       </c>
       <c r="E15">
@@ -7145,7 +7144,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -7155,7 +7154,7 @@
       <c r="C16" t="s">
         <v>149</v>
       </c>
-      <c r="D16" s="11">
+      <c r="D16">
         <v>911</v>
       </c>
       <c r="E16">
@@ -7165,7 +7164,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -7175,7 +7174,7 @@
       <c r="C17" t="s">
         <v>353</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17">
         <v>932</v>
       </c>
       <c r="E17">
@@ -7185,7 +7184,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -7195,7 +7194,7 @@
       <c r="C18" t="s">
         <v>155</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18">
         <v>933</v>
       </c>
       <c r="E18">
@@ -7205,7 +7204,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -7215,7 +7214,7 @@
       <c r="C19" t="s">
         <v>352</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19">
         <v>931</v>
       </c>
       <c r="E19">
@@ -7225,7 +7224,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -7235,7 +7234,7 @@
       <c r="C20" t="s">
         <v>150</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20">
         <v>925</v>
       </c>
       <c r="E20">
@@ -7245,7 +7244,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -7255,7 +7254,7 @@
       <c r="C21" t="s">
         <v>137</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21">
         <v>943</v>
       </c>
       <c r="E21">
@@ -7265,7 +7264,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -7275,7 +7274,7 @@
       <c r="C22" t="s">
         <v>125</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22">
         <v>812</v>
       </c>
       <c r="E22">
@@ -7285,7 +7284,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -7305,7 +7304,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -7325,7 +7324,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -7345,7 +7344,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -7365,7 +7364,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -7385,45 +7384,45 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="11">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>24</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" t="s">
         <v>266</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" t="s">
         <v>122</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
-      <c r="F28" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="G28" s="11" t="s">
+      <c r="F28" t="s">
+        <v>40</v>
+      </c>
+      <c r="G28" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="11">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>25</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" t="s">
         <v>267</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" t="s">
         <v>123</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
-      <c r="F29" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="G29" s="11" t="s">
+      <c r="F29" t="s">
+        <v>40</v>
+      </c>
+      <c r="G29" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>26</v>
       </c>
@@ -7443,8 +7442,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B31" s="14" t="s">
+    <row r="31" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B31" s="13" t="s">
         <v>329</v>
       </c>
       <c r="C31" s="7"/>
@@ -7454,7 +7453,7 @@
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>27</v>
       </c>
@@ -7473,7 +7472,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>28</v>
       </c>
@@ -7492,7 +7491,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>29</v>
       </c>
@@ -7513,7 +7512,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>30</v>
       </c>
@@ -7533,7 +7532,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>31</v>
       </c>
@@ -7556,7 +7555,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>32</v>
       </c>
@@ -7579,7 +7578,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>33</v>
       </c>
@@ -7599,7 +7598,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>34</v>
       </c>
@@ -7622,7 +7621,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>35</v>
       </c>
@@ -7645,7 +7644,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>36</v>
       </c>
@@ -7668,7 +7667,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>37</v>
       </c>
@@ -7688,18 +7687,18 @@
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B43" s="15" t="s">
+    <row r="43" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B43" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="C43" s="16"/>
-      <c r="D43" s="16"/>
-      <c r="E43" s="16"/>
-      <c r="F43" s="16"/>
-      <c r="G43" s="16"/>
-      <c r="H43" s="16"/>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>38</v>
       </c>
@@ -7719,7 +7718,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>39</v>
       </c>
@@ -7739,7 +7738,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>40</v>
       </c>
@@ -7759,7 +7758,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>41</v>
       </c>
@@ -7779,7 +7778,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>42</v>
       </c>
@@ -7802,7 +7801,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>43</v>
       </c>
@@ -7825,7 +7824,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>44</v>
       </c>
@@ -7845,7 +7844,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>45</v>
       </c>
@@ -7865,7 +7864,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>46</v>
       </c>
@@ -7895,14 +7894,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BC90879-45EA-46D4-957C-588B6196CFF5}">
   <dimension ref="A1:F47"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="38.44140625" customWidth="1"/>
+    <col min="2" max="2" width="38.42578125" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>372</v>
       </c>
@@ -7922,14 +7921,14 @@
         <v>339</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>201</v>
       </c>
       <c r="B2" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="11">
+      <c r="C2">
         <v>210</v>
       </c>
       <c r="D2">
@@ -7939,14 +7938,14 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>202</v>
       </c>
       <c r="B3" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3">
         <v>220</v>
       </c>
       <c r="D3">
@@ -7956,14 +7955,14 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>208</v>
       </c>
       <c r="B4" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4">
         <v>252</v>
       </c>
       <c r="D4">
@@ -7973,14 +7972,14 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>209</v>
       </c>
       <c r="B5" t="s">
         <v>65</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5">
         <v>253</v>
       </c>
       <c r="D5">
@@ -7990,7 +7989,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>211</v>
       </c>
@@ -8007,7 +8006,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>214</v>
       </c>
@@ -8024,7 +8023,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>205</v>
       </c>
@@ -8041,14 +8040,14 @@
         <v>344</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>169</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9">
         <v>820</v>
       </c>
       <c r="D9">
@@ -8058,14 +8057,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>292</v>
       </c>
       <c r="B10" t="s">
         <v>148</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10">
         <v>890</v>
       </c>
       <c r="D10">
@@ -8075,14 +8074,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>290</v>
       </c>
       <c r="B11" t="s">
         <v>146</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11">
         <v>880</v>
       </c>
       <c r="D11">
@@ -8092,14 +8091,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>283</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12">
         <v>850</v>
       </c>
       <c r="D12">
@@ -8109,14 +8108,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>293</v>
       </c>
       <c r="B13" t="s">
         <v>149</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13">
         <v>911</v>
       </c>
       <c r="D13">
@@ -8126,14 +8125,14 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>298</v>
       </c>
       <c r="B14" t="s">
         <v>353</v>
       </c>
-      <c r="C14" s="11">
+      <c r="C14">
         <v>932</v>
       </c>
       <c r="D14">
@@ -8143,14 +8142,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>299</v>
       </c>
       <c r="B15" t="s">
         <v>155</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15">
         <v>933</v>
       </c>
       <c r="D15">
@@ -8160,14 +8159,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>297</v>
       </c>
       <c r="B16" t="s">
         <v>352</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16">
         <v>931</v>
       </c>
       <c r="D16">
@@ -8177,14 +8176,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>294</v>
       </c>
       <c r="B17" t="s">
         <v>150</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17">
         <v>925</v>
       </c>
       <c r="D17">
@@ -8194,14 +8193,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>280</v>
       </c>
       <c r="B18" t="s">
         <v>137</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18">
         <v>943</v>
       </c>
       <c r="D18">
@@ -8211,14 +8210,14 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>268</v>
       </c>
       <c r="B19" t="s">
         <v>125</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19">
         <v>812</v>
       </c>
       <c r="D19">
@@ -8228,7 +8227,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>270</v>
       </c>
@@ -8245,7 +8244,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>254</v>
       </c>
@@ -8262,7 +8261,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>258</v>
       </c>
@@ -8279,7 +8278,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>184</v>
       </c>
@@ -8296,7 +8295,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>186</v>
       </c>
@@ -8313,39 +8312,39 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>266</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" t="s">
         <v>122</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F25" s="11" t="s">
+      <c r="E25" t="s">
+        <v>40</v>
+      </c>
+      <c r="F25" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="26" spans="1:6" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>267</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" t="s">
         <v>123</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
-      <c r="E26" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F26" s="11" t="s">
+      <c r="E26" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>277</v>
       </c>
@@ -8362,7 +8361,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>216</v>
       </c>
@@ -8378,7 +8377,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>326</v>
       </c>
@@ -8394,7 +8393,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>221</v>
       </c>
@@ -8410,7 +8409,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>222</v>
       </c>
@@ -8427,7 +8426,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>223</v>
       </c>
@@ -8447,7 +8446,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>224</v>
       </c>
@@ -8467,7 +8466,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>225</v>
       </c>
@@ -8484,7 +8483,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>226</v>
       </c>
@@ -8504,7 +8503,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>227</v>
       </c>
@@ -8524,7 +8523,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>232</v>
       </c>
@@ -8544,7 +8543,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>234</v>
       </c>
@@ -8561,7 +8560,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>243</v>
       </c>
@@ -8578,7 +8577,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>237</v>
       </c>
@@ -8595,7 +8594,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>236</v>
       </c>
@@ -8612,7 +8611,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>235</v>
       </c>
@@ -8629,7 +8628,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>239</v>
       </c>
@@ -8649,7 +8648,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>244</v>
       </c>
@@ -8666,7 +8665,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>247</v>
       </c>
@@ -8683,7 +8682,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>249</v>
       </c>
@@ -8700,7 +8699,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>250</v>
       </c>
@@ -8725,13 +8724,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A244719-B145-49E2-B26D-5AE8DB9D4751}">
-  <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="41.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>372</v>
       </c>
@@ -8751,7 +8750,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>201</v>
       </c>
@@ -8768,7 +8767,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>202</v>
       </c>
@@ -8785,7 +8784,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>208</v>
       </c>
@@ -8802,7 +8801,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>209</v>
       </c>
@@ -8819,7 +8818,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>211</v>
       </c>
@@ -8836,7 +8835,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>214</v>
       </c>
@@ -8853,7 +8852,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>205</v>
       </c>
@@ -8870,7 +8869,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>169</v>
       </c>
@@ -8887,7 +8886,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>292</v>
       </c>
@@ -8904,7 +8903,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>290</v>
       </c>
@@ -8921,7 +8920,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>283</v>
       </c>
@@ -8938,7 +8937,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>293</v>
       </c>
@@ -8955,7 +8954,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>298</v>
       </c>
@@ -8972,7 +8971,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>299</v>
       </c>
@@ -8989,7 +8988,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>297</v>
       </c>
@@ -9006,7 +9005,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>294</v>
       </c>
@@ -9023,7 +9022,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>280</v>
       </c>
@@ -9040,7 +9039,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>268</v>
       </c>
@@ -9057,7 +9056,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>270</v>
       </c>
@@ -9074,7 +9073,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>254</v>
       </c>
@@ -9091,7 +9090,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>258</v>
       </c>
@@ -9108,7 +9107,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>184</v>
       </c>
@@ -9125,7 +9124,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>186</v>
       </c>
@@ -9142,7 +9141,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>222</v>
       </c>
@@ -9159,293 +9158,273 @@
         <v>333</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B26" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C26">
-        <v>416</v>
+        <v>420</v>
       </c>
       <c r="D26">
-        <v>12.57</v>
+        <v>2.41</v>
       </c>
       <c r="E26" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F26" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>225</v>
+      </c>
+      <c r="B27" t="s">
+        <v>81</v>
+      </c>
+      <c r="C27">
+        <v>430</v>
+      </c>
+      <c r="D27">
+        <v>30.38</v>
+      </c>
+      <c r="E27" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>226</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="C28">
+        <v>437</v>
+      </c>
+      <c r="D28">
+        <v>1.48</v>
+      </c>
+      <c r="E28" t="s">
+        <v>375</v>
+      </c>
+      <c r="F28" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>224</v>
-      </c>
-      <c r="B27" t="s">
-        <v>80</v>
-      </c>
-      <c r="C27">
-        <v>420</v>
-      </c>
-      <c r="D27">
-        <v>2.41</v>
-      </c>
-      <c r="E27" t="s">
-        <v>338</v>
-      </c>
-      <c r="F27" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>227</v>
+      </c>
+      <c r="B29" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29">
+        <v>444</v>
+      </c>
+      <c r="D29">
+        <v>220</v>
+      </c>
+      <c r="E29" t="s">
+        <v>376</v>
+      </c>
+      <c r="F29" t="s">
         <v>345</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>225</v>
-      </c>
-      <c r="B28" t="s">
-        <v>81</v>
-      </c>
-      <c r="C28">
-        <v>430</v>
-      </c>
-      <c r="D28">
-        <v>30.38</v>
-      </c>
-      <c r="E28" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>226</v>
-      </c>
-      <c r="B29" t="s">
-        <v>82</v>
-      </c>
-      <c r="C29">
-        <v>437</v>
-      </c>
-      <c r="D29">
-        <v>1.48</v>
-      </c>
-      <c r="E29" t="s">
-        <v>375</v>
-      </c>
-      <c r="F29" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>232</v>
+      </c>
+      <c r="B30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30">
+        <v>492</v>
+      </c>
+      <c r="D30">
+        <v>38.97</v>
+      </c>
+      <c r="E30" t="s">
+        <v>44</v>
+      </c>
+      <c r="F30" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>227</v>
-      </c>
-      <c r="B30" t="s">
-        <v>83</v>
-      </c>
-      <c r="C30">
-        <v>444</v>
-      </c>
-      <c r="D30">
-        <v>220</v>
-      </c>
-      <c r="E30" t="s">
-        <v>376</v>
-      </c>
-      <c r="F30" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B31" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C31">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="D31">
-        <v>38.97</v>
+        <v>28.82</v>
       </c>
       <c r="E31" t="s">
         <v>44</v>
       </c>
-      <c r="F31" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
       <c r="B32" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C32">
-        <v>495</v>
+        <v>550</v>
       </c>
       <c r="D32">
-        <v>28.82</v>
+        <v>1.56</v>
       </c>
       <c r="E32" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B33" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C33">
-        <v>550</v>
+        <v>530</v>
       </c>
       <c r="D33">
-        <v>1.56</v>
+        <v>2.0299999999999998</v>
       </c>
       <c r="E33" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B34" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C34">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="D34">
-        <v>2.0299999999999998</v>
+        <v>2.13</v>
       </c>
       <c r="E34" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C35">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D35">
-        <v>2.13</v>
+        <v>1.89</v>
       </c>
       <c r="E35" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>351</v>
       </c>
       <c r="C36">
-        <v>520</v>
+        <v>536</v>
       </c>
       <c r="D36">
-        <v>1.89</v>
+        <v>2.48</v>
       </c>
       <c r="E36" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F36" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B37" t="s">
-        <v>351</v>
+        <v>100</v>
       </c>
       <c r="C37">
-        <v>536</v>
+        <v>560</v>
       </c>
       <c r="D37">
-        <v>2.48</v>
+        <v>9.9</v>
       </c>
       <c r="E37" t="s">
-        <v>46</v>
-      </c>
-      <c r="F37" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B38" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C38">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="D38">
-        <v>9.9</v>
+        <v>47.62</v>
       </c>
       <c r="E38" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B39" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C39">
-        <v>565</v>
+        <v>590</v>
       </c>
       <c r="D39">
-        <v>47.62</v>
+        <v>72.05</v>
       </c>
       <c r="E39" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B40" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C40">
-        <v>590</v>
+        <v>610</v>
       </c>
       <c r="D40">
-        <v>72.05</v>
+        <v>10.723000000000001</v>
       </c>
       <c r="E40" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>250</v>
-      </c>
-      <c r="B41" t="s">
-        <v>106</v>
-      </c>
-      <c r="C41">
-        <v>610</v>
-      </c>
-      <c r="D41">
-        <v>10.723000000000001</v>
-      </c>
-      <c r="E41" t="s">
         <v>44</v>
       </c>
     </row>
@@ -9457,13 +9436,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2FFD004-89BD-4461-90DD-23940889AC29}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="73.33203125" customWidth="1"/>
+    <col min="1" max="1" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="73.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>339</v>
       </c>
@@ -9471,27 +9450,27 @@
         <v>355</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
+    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="18" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
         <v>358</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="18" t="s">
         <v>359</v>
       </c>
     </row>
@@ -9503,13 +9482,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF9160ED-ADEC-4EC7-AF5D-CA210C03965A}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" customWidth="1"/>
-    <col min="2" max="2" width="24.5546875" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>346</v>
       </c>
@@ -9520,7 +9499,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>333</v>
       </c>
@@ -9531,7 +9510,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>338</v>
       </c>
@@ -9542,7 +9521,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -9553,7 +9532,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -9564,7 +9543,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>335</v>
       </c>
@@ -9575,7 +9554,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>344</v>
       </c>
@@ -9594,22 +9573,22 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE2F8E74-9EA0-439D-8AB3-EB1BD26461D1}">
   <dimension ref="A1:U51"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="3" max="3" width="38.44140625" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="3" max="3" width="38.42578125" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" customWidth="1"/>
     <col min="7" max="7" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="F1" t="s">
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B2" s="18" t="s">
+    <row r="2" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B2" s="17" t="s">
         <v>331</v>
       </c>
       <c r="C2" s="3"/>
@@ -9618,7 +9597,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -9647,7 +9626,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -9676,7 +9655,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -9705,7 +9684,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -9734,8 +9713,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B7" s="12" t="s">
+    <row r="7" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B7" s="11" t="s">
         <v>327</v>
       </c>
       <c r="C7" s="5"/>
@@ -9744,7 +9723,7 @@
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5</v>
       </c>
@@ -9773,7 +9752,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>6</v>
       </c>
@@ -9802,8 +9781,8 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B10" s="13" t="s">
+    <row r="10" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B10" s="12" t="s">
         <v>328</v>
       </c>
       <c r="C10" s="9"/>
@@ -9812,7 +9791,7 @@
       <c r="F10" s="9"/>
       <c r="G10" s="9"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>7</v>
       </c>
@@ -9844,7 +9823,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>8</v>
       </c>
@@ -9873,7 +9852,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9</v>
       </c>
@@ -9902,7 +9881,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -9931,7 +9910,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>11</v>
       </c>
@@ -9960,7 +9939,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>12</v>
       </c>
@@ -9989,7 +9968,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>13</v>
       </c>
@@ -10018,7 +9997,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>14</v>
       </c>
@@ -10047,7 +10026,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15</v>
       </c>
@@ -10076,7 +10055,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>16</v>
       </c>
@@ -10105,7 +10084,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>17</v>
       </c>
@@ -10134,7 +10113,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>18</v>
       </c>
@@ -10163,7 +10142,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>19</v>
       </c>
@@ -10192,7 +10171,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>20</v>
       </c>
@@ -10221,7 +10200,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>21</v>
       </c>
@@ -10250,7 +10229,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>22</v>
       </c>
@@ -10279,7 +10258,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>23</v>
       </c>
@@ -10297,7 +10276,7 @@
       </c>
       <c r="L27" s="10"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>24</v>
       </c>
@@ -10315,7 +10294,7 @@
       </c>
       <c r="L28" s="10"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>25</v>
       </c>
@@ -10344,8 +10323,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="B30" s="14" t="s">
+    <row r="30" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B30" s="13" t="s">
         <v>329</v>
       </c>
       <c r="C30" s="7"/>
@@ -10354,7 +10333,7 @@
       <c r="F30" s="7"/>
       <c r="G30" s="7"/>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>26</v>
       </c>
@@ -10372,7 +10351,7 @@
       </c>
       <c r="L31" s="10"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>27</v>
       </c>
@@ -10390,7 +10369,7 @@
       </c>
       <c r="L32" s="10"/>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>28</v>
       </c>
@@ -10411,7 +10390,7 @@
       </c>
       <c r="L33" s="10"/>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>29</v>
       </c>
@@ -10440,7 +10419,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>30</v>
       </c>
@@ -10491,7 +10470,7 @@
         <v>17.219178082191782</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>31</v>
       </c>
@@ -10535,7 +10514,7 @@
         <v>2.41</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>32</v>
       </c>
@@ -10564,7 +10543,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>33</v>
       </c>
@@ -10615,7 +10594,7 @@
         <v>24.436548223350254</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>34</v>
       </c>
@@ -10665,7 +10644,7 @@
         <v>78.09</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>35</v>
       </c>
@@ -10710,7 +10689,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>36</v>
       </c>
@@ -10749,17 +10728,17 @@
         <v>16.375</v>
       </c>
     </row>
-    <row r="42" spans="1:21" ht="18" x14ac:dyDescent="0.35">
-      <c r="B42" s="15" t="s">
+    <row r="42" spans="1:21" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B42" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="16"/>
-      <c r="E42" s="16"/>
-      <c r="F42" s="16"/>
-      <c r="G42" s="16"/>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+    </row>
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>37</v>
       </c>
@@ -10788,7 +10767,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>38</v>
       </c>
@@ -10826,7 +10805,7 @@
         <v>6.4689655172413802</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>39</v>
       </c>
@@ -10861,7 +10840,7 @@
         <v>16.949579831932777</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>40</v>
       </c>
@@ -10899,7 +10878,7 @@
         <v>4.6810551558753</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>41</v>
       </c>
@@ -10940,7 +10919,7 @@
         <v>9.3665335016831524</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>42</v>
       </c>
@@ -10989,7 +10968,7 @@
         <v>9.9042857142857148</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>43</v>
       </c>
@@ -11018,7 +10997,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>44</v>
       </c>
@@ -11047,7 +11026,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>45</v>
       </c>

</xml_diff>